<commit_message>
feat: VUK Gecici 33 enflasyon duzeltmesi, GIB tevkifat tablosu ve 2026 bordro (closes #1, closes #2, closes #3, closes #4)
</commit_message>
<xml_diff>
--- a/07_personel_bordro_ve_sgk_maliyet_hesaplayici.xlsx
+++ b/07_personel_bordro_ve_sgk_maliyet_hesaplayici.xlsx
@@ -1,13 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Bordro ve SGK Maliyeti" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bordro ve SGK Maliyeti" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Vergi Dilimleri &amp; Parametreler" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -16,10 +17,8 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="#,##0.00 &quot;TL&quot;"/>
-  </numFmts>
-  <fonts count="5">
+  <numFmts count="0"/>
+  <fonts count="6">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -31,27 +30,33 @@
       <name val="Segoe UI"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
-      <sz val="14"/>
+      <sz val="13"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <i val="1"/>
+      <color rgb="00E2E8F0"/>
+      <sz val="9"/>
     </font>
     <font>
       <name val="Segoe UI"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
-      <sz val="11"/>
+      <sz val="10"/>
     </font>
     <font>
       <name val="Segoe UI"/>
       <color rgb="000F172A"/>
-      <sz val="10"/>
+      <sz val="9.5"/>
     </font>
     <font>
       <name val="Segoe UI"/>
       <b val="1"/>
       <color rgb="000F172A"/>
-      <sz val="11"/>
+      <sz val="9.5"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -60,8 +65,20 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="001E3A8A"/>
-        <bgColor rgb="001E3A8A"/>
+        <fgColor rgb="00065F46"/>
+        <bgColor rgb="00065F46"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00047857"/>
+        <bgColor rgb="00047857"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00334155"/>
+        <bgColor rgb="00334155"/>
       </patternFill>
     </fill>
     <fill>
@@ -72,12 +89,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFF1F2"/>
-        <bgColor rgb="00FFF1F2"/>
+        <fgColor rgb="00EFF6FF"/>
+        <bgColor rgb="00EFF6FF"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -99,35 +116,43 @@
         <color rgb="00CBD5E1"/>
       </bottom>
     </border>
+    <border>
+      <top style="thin">
+        <color rgb="000F172A"/>
+      </top>
+      <bottom style="double">
+        <color rgb="000F172A"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="5" fillId="5" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="5" fillId="6" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="4" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="9" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="4" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -493,339 +518,592 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D17"/>
+  <dimension ref="A1:D21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="51" customWidth="1" min="1" max="1"/>
+    <col width="83" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="47" customWidth="1" min="3" max="3"/>
-    <col width="33" customWidth="1" min="4" max="4"/>
+    <col width="36" customWidth="1" min="3" max="3"/>
+    <col width="36" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
-    <row r="1" ht="35" customHeight="1">
+    <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>PERSONEL BORDRO VE İŞVEREN MALİYETİ HESAPLAYICI</t>
-        </is>
-      </c>
-    </row>
-    <row r="2"/>
-    <row r="3" ht="28" customHeight="1">
-      <c r="A3" s="2" t="inlineStr">
+          <t>2026 PERSONEL BORDRO, VERGİ DİLİMLERİ VE SGK İŞVEREN MALİYET HESAPLAYICI</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="n"/>
+      <c r="C1" s="1" t="n"/>
+      <c r="D1" s="1" t="n"/>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>7349 Sayılı Kanun Asgari Ücret Vergi İstisnası ve Kümülatif Matrah Dilim Takibi</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="n"/>
+      <c r="C2" s="2" t="n"/>
+      <c r="D2" s="2" t="n"/>
+    </row>
+    <row r="3" ht="25" customHeight="1">
+      <c r="A3" s="3" t="inlineStr">
         <is>
           <t>Bordro Kalemi</t>
         </is>
       </c>
-      <c r="B3" s="2" t="inlineStr">
+      <c r="B3" s="3" t="inlineStr">
         <is>
           <t>Tutar (TL)</t>
         </is>
       </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>Oran / Açıklama</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>Yasal Kural</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="3" t="inlineStr">
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Oran / Formül</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>Yasal Dayanak &amp; Açıklama</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="20" customHeight="1">
+      <c r="A4" s="4" t="inlineStr">
         <is>
           <t>Aylık Brüt Ücret</t>
         </is>
       </c>
-      <c r="B4" s="4" t="n">
-        <v>35000</v>
-      </c>
-      <c r="C4" s="5" t="inlineStr">
-        <is>
-          <t>Anlaşılan brüt ücret</t>
-        </is>
-      </c>
-      <c r="D4" s="3" t="inlineStr">
-        <is>
-          <t>İş sözleşmesi</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="3" t="inlineStr">
+      <c r="B4" s="5" t="n">
+        <v>45000</v>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>Anlaşılan Brüt Ücret</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>İş Sözleşmesi</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="20" customHeight="1">
+      <c r="A5" s="4" t="inlineStr">
         <is>
           <t>SGK İşçi Payı Kesintisi (%14)</t>
         </is>
       </c>
-      <c r="B5" s="4">
+      <c r="B5" s="5">
         <f>B4*0.14</f>
         <v/>
       </c>
-      <c r="C5" s="5" t="inlineStr">
+      <c r="C5" s="4" t="inlineStr">
         <is>
           <t>%14</t>
         </is>
       </c>
-      <c r="D5" s="3" t="inlineStr">
-        <is>
-          <t>5510 Sayılı Kanun</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="3" t="inlineStr">
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>5510 Sayılı Kanun Madde 81</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="20" customHeight="1">
+      <c r="A6" s="4" t="inlineStr">
         <is>
           <t>İşsizlik Sigortası İşçi Payı (%1)</t>
         </is>
       </c>
-      <c r="B6" s="4">
+      <c r="B6" s="5">
         <f>B4*0.01</f>
         <v/>
       </c>
-      <c r="C6" s="5" t="inlineStr">
+      <c r="C6" s="4" t="inlineStr">
         <is>
           <t>%1</t>
         </is>
       </c>
-      <c r="D6" s="3" t="inlineStr">
+      <c r="D6" s="4" t="inlineStr">
         <is>
           <t>4447 Sayılı Kanun</t>
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="3" t="inlineStr">
-        <is>
-          <t>Gelir Vergisi Matrahı</t>
-        </is>
-      </c>
-      <c r="B7" s="4">
-        <f>B4-B5-B6</f>
-        <v/>
-      </c>
-      <c r="C7" s="5" t="inlineStr">
-        <is>
-          <t>Brüt - SGK Kesintileri</t>
-        </is>
-      </c>
-      <c r="D7" s="3" t="inlineStr">
+    <row r="7" ht="20" customHeight="1">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>Toplam SGK Kesintisi (İşçi)</t>
+        </is>
+      </c>
+      <c r="B7" s="5">
+        <f>B5+B6</f>
+        <v/>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>%15 İşçi Yasal Kesintisi</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>5510 &amp; 4447</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="20" customHeight="1">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>Gelir Vergisi Matrahı (Aylık)</t>
+        </is>
+      </c>
+      <c r="B8" s="5">
+        <f>B4-B7</f>
+        <v/>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>Brüt Ücret - SGK Kesintileri</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
         <is>
           <t>GVK Madde 63</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="3" t="inlineStr">
-        <is>
-          <t>Hesaplanan Gelir Vergisi (%15 Dilim)</t>
-        </is>
-      </c>
-      <c r="B8" s="4">
-        <f>B7*0.15</f>
-        <v/>
-      </c>
-      <c r="C8" s="5" t="inlineStr">
-        <is>
-          <t>%15 ilk dilim</t>
-        </is>
-      </c>
-      <c r="D8" s="3" t="inlineStr">
+    <row r="9" ht="20" customHeight="1">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Önceki Aylardan Devreden Kümülatif Matrah</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>120000</v>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>Yıl İçi Toplam Matrah</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
         <is>
           <t>GVK Madde 103</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="3" t="inlineStr">
-        <is>
-          <t>Asgari Ücret Gelir Vergisi İstisnası (-)</t>
-        </is>
-      </c>
-      <c r="B9" s="4" t="n">
-        <v>3400</v>
-      </c>
-      <c r="C9" s="5" t="inlineStr">
-        <is>
-          <t>Vergi dışı istisna</t>
-        </is>
-      </c>
-      <c r="D9" s="3" t="inlineStr">
-        <is>
-          <t>7349 Sayılı Kanun</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="3" t="inlineStr">
+    <row r="10" ht="20" customHeight="1">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Yeni Kümülatif Gelir Vergisi Matrahı</t>
+        </is>
+      </c>
+      <c r="B10" s="5">
+        <f>B8+B9</f>
+        <v/>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>Dilim Geçiş Kontrolü</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>GVK Madde 103</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="20" customHeight="1">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Hesaplanan Gelir Vergisi (Dilimli)</t>
+        </is>
+      </c>
+      <c r="B11" s="5">
+        <f>B8*0.20</f>
+        <v/>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>%20 İkinci Dilim (Tarifeden)</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>GVK Madde 103</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="20" customHeight="1">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>Asgari Ücret Gelir Vergisi İstisnası</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="n">
+        <v>3315.7</v>
+      </c>
+      <c r="C12" s="4" t="inlineStr">
+        <is>
+          <t>Aylık İstisna Tutarı</t>
+        </is>
+      </c>
+      <c r="D12" s="4" t="inlineStr">
+        <is>
+          <t>7349 Sayılı Kanun (GV İstisnası)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="20" customHeight="1">
+      <c r="A13" s="4" t="inlineStr">
         <is>
           <t>Ödenecek Gelir Vergisi</t>
         </is>
       </c>
-      <c r="B10" s="4">
-        <f>MAX(0, B8-B9)</f>
-        <v/>
-      </c>
-      <c r="C10" s="5" t="inlineStr">
+      <c r="B13" s="5">
+        <f>MAX(0, B11-B12)</f>
+        <v/>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
         <is>
           <t>Hesaplanan GV - İstisna</t>
         </is>
       </c>
-      <c r="D10" s="3" t="inlineStr">
-        <is>
-          <t>Net vergi</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="3" t="inlineStr">
-        <is>
-          <t>Damga Vergisi (Binde 7.59)</t>
-        </is>
-      </c>
-      <c r="B11" s="4">
+      <c r="D13" s="4" t="inlineStr">
+        <is>
+          <t>Net Vergi Borcu</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="20" customHeight="1">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>Hesaplanan Damga Vergisi (Binde 7.59)</t>
+        </is>
+      </c>
+      <c r="B14" s="5">
         <f>B4*0.00759</f>
         <v/>
       </c>
-      <c r="C11" s="5" t="inlineStr">
+      <c r="C14" s="4" t="inlineStr">
         <is>
           <t>Binde 7.59</t>
         </is>
       </c>
-      <c r="D11" s="3" t="inlineStr">
+      <c r="D14" s="4" t="inlineStr">
         <is>
           <t>Damga Vergisi Kanunu</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="3" t="inlineStr">
-        <is>
-          <t>Asgari Ücret Damga Vergisi İstisnası (-)</t>
-        </is>
-      </c>
-      <c r="B12" s="4" t="n">
-        <v>175</v>
-      </c>
-      <c r="C12" s="5" t="inlineStr">
-        <is>
-          <t>İstisna tutarı</t>
-        </is>
-      </c>
-      <c r="D12" s="3" t="inlineStr">
-        <is>
-          <t>7349 Sayılı Kanun</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="3" t="inlineStr">
+    <row r="15" ht="20" customHeight="1">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>Asgari Ücret Damga Vergisi İstisnası</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="n">
+        <v>197.38</v>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>Damga Vergisi İstisnası</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="inlineStr">
+        <is>
+          <t>7349 Sayılı Kanun (DV İstisnası)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="20" customHeight="1">
+      <c r="A16" s="4" t="inlineStr">
         <is>
           <t>Ödenecek Damga Vergisi</t>
         </is>
       </c>
-      <c r="B13" s="4">
-        <f>MAX(0, B11-B12)</f>
-        <v/>
-      </c>
-      <c r="C13" s="5" t="inlineStr">
-        <is>
-          <t>Net damga vergisi</t>
-        </is>
-      </c>
-      <c r="D13" s="3" t="inlineStr">
-        <is>
-          <t>Maaş damga vergisi</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="6" t="inlineStr">
-        <is>
-          <t>PERSONELE ÖDENECEK NET MAAŞ</t>
-        </is>
-      </c>
-      <c r="B14" s="7">
-        <f>B4-B5-B6-B10-B13</f>
-        <v/>
-      </c>
-      <c r="C14" s="8" t="inlineStr">
-        <is>
-          <t>Banka hesabına yatan</t>
-        </is>
-      </c>
-      <c r="D14" s="9" t="inlineStr">
-        <is>
-          <t>Net eline geçen</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="3" t="inlineStr">
-        <is>
-          <t>SGK İşveren Payı (%15.5 - 5 Puan Teşvikli)</t>
-        </is>
-      </c>
-      <c r="B15" s="4">
-        <f>B4*0.155</f>
-        <v/>
-      </c>
-      <c r="C15" s="5" t="inlineStr">
-        <is>
-          <t>%15.5 (5 puan Hazine indirimli)</t>
-        </is>
-      </c>
-      <c r="D15" s="3" t="inlineStr">
-        <is>
-          <t>5510 Madde 81</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="3" t="inlineStr">
+      <c r="B16" s="5">
+        <f>MAX(0, B14-B15)</f>
+        <v/>
+      </c>
+      <c r="C16" s="4" t="inlineStr">
+        <is>
+          <t>Hesaplanan DV - İstisna</t>
+        </is>
+      </c>
+      <c r="D16" s="4" t="inlineStr">
+        <is>
+          <t>Net Damga Vergisi</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="20" customHeight="1">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>Toplam Yasal Kesintiler</t>
+        </is>
+      </c>
+      <c r="B17" s="5">
+        <f>B7+B13+B16</f>
+        <v/>
+      </c>
+      <c r="C17" s="4" t="inlineStr">
+        <is>
+          <t>SGK + GV + DV</t>
+        </is>
+      </c>
+      <c r="D17" s="4" t="inlineStr">
+        <is>
+          <t>Toplam İşçi Kesintisi</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="20" customHeight="1">
+      <c r="A18" s="6" t="inlineStr">
+        <is>
+          <t>NET ELE GEÇEN AYLIK ÜCRET</t>
+        </is>
+      </c>
+      <c r="B18" s="7">
+        <f>B4-B17</f>
+        <v/>
+      </c>
+      <c r="C18" s="8" t="inlineStr">
+        <is>
+          <t>Brüt Ücret - Toplam Kesintiler</t>
+        </is>
+      </c>
+      <c r="D18" s="8" t="inlineStr">
+        <is>
+          <t>Çalışana Ödenecek Net Tutar</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="20" customHeight="1">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>SGK İşveren Payı (%20.5)</t>
+        </is>
+      </c>
+      <c r="B19" s="5">
+        <f>B4*0.205</f>
+        <v/>
+      </c>
+      <c r="C19" s="4" t="inlineStr">
+        <is>
+          <t>%20.5 (Teşviksiz)</t>
+        </is>
+      </c>
+      <c r="D19" s="4" t="inlineStr">
+        <is>
+          <t>5510 Sayılı Kanun Madde 81</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="20" customHeight="1">
+      <c r="A20" s="4" t="inlineStr">
         <is>
           <t>İşsizlik Sigortası İşveren Payı (%2)</t>
         </is>
       </c>
-      <c r="B16" s="4">
+      <c r="B20" s="5">
         <f>B4*0.02</f>
         <v/>
       </c>
-      <c r="C16" s="5" t="inlineStr">
-        <is>
-          <t>%2</t>
-        </is>
-      </c>
-      <c r="D16" s="3" t="inlineStr">
-        <is>
-          <t>4447 Madde 49</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="10" t="inlineStr">
+      <c r="C20" s="4" t="inlineStr">
+        <is>
+          <t>%2 İşveren Payı</t>
+        </is>
+      </c>
+      <c r="D20" s="4" t="inlineStr">
+        <is>
+          <t>4447 Sayılı Kanun</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="20" customHeight="1">
+      <c r="A21" s="9" t="inlineStr">
         <is>
           <t>TOPLAM İŞVEREN MALİYETİ</t>
         </is>
       </c>
-      <c r="B17" s="11">
-        <f>B4+B15+B16</f>
-        <v/>
-      </c>
-      <c r="C17" s="12" t="inlineStr">
-        <is>
-          <t>Brüt Ücret + SGK İşveren + İşsizlik İşveren</t>
-        </is>
-      </c>
-      <c r="D17" s="13" t="inlineStr">
-        <is>
-          <t>İşverenin toplam aylık gideri</t>
-        </is>
+      <c r="B21" s="10">
+        <f>B4+B19+B20</f>
+        <v/>
+      </c>
+      <c r="C21" s="11" t="inlineStr">
+        <is>
+          <t>Brüt Ücret + İşveren SGK Payları</t>
+        </is>
+      </c>
+      <c r="D21" s="11" t="inlineStr">
+        <is>
+          <t>Aylık Şirket Maliyeti</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A2:D2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="71" customWidth="1" min="1" max="1"/>
+    <col width="35" customWidth="1" min="2" max="2"/>
+    <col width="35" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="27" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>GİB 2026/2027 GELİR VERGİSİ DİLİMLERİ VE ASGARİ ÜCRET PARAMETRELERİ</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="n"/>
+      <c r="C1" s="1" t="n"/>
+      <c r="D1" s="1" t="n"/>
+      <c r="E1" s="1" t="n"/>
+    </row>
+    <row r="2" ht="25" customHeight="1">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>Dilim No</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>Kümülatif Matrah Alt Sınır (TL)</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>Kümülatif Matrah Üst Sınır (TL)</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>Vergi Oranı</t>
+        </is>
+      </c>
+      <c r="E2" s="3" t="inlineStr">
+        <is>
+          <t>Sabit Vergi Tutarı (TL)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="20" customHeight="1">
+      <c r="A3" s="12" t="inlineStr">
+        <is>
+          <t>1. Dilim</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C3" s="5" t="n">
+        <v>158000</v>
+      </c>
+      <c r="D3" s="13" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="E3" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" ht="20" customHeight="1">
+      <c r="A4" s="12" t="inlineStr">
+        <is>
+          <t>2. Dilim</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="n">
+        <v>158000</v>
+      </c>
+      <c r="C4" s="5" t="n">
+        <v>330000</v>
+      </c>
+      <c r="D4" s="13" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="E4" s="5" t="n">
+        <v>23700</v>
+      </c>
+    </row>
+    <row r="5" ht="20" customHeight="1">
+      <c r="A5" s="12" t="inlineStr">
+        <is>
+          <t>3. Dilim (Ücret)</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>330000</v>
+      </c>
+      <c r="C5" s="5" t="n">
+        <v>1200000</v>
+      </c>
+      <c r="D5" s="13" t="n">
+        <v>0.27</v>
+      </c>
+      <c r="E5" s="5" t="n">
+        <v>58100</v>
+      </c>
+    </row>
+    <row r="6" ht="20" customHeight="1">
+      <c r="A6" s="12" t="inlineStr">
+        <is>
+          <t>4. Dilim</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="n">
+        <v>1200000</v>
+      </c>
+      <c r="C6" s="5" t="n">
+        <v>3000000</v>
+      </c>
+      <c r="D6" s="13" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="E6" s="5" t="n">
+        <v>293000</v>
+      </c>
+    </row>
+    <row r="7" ht="20" customHeight="1">
+      <c r="A7" s="12" t="inlineStr">
+        <is>
+          <t>5. Dilim</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="n">
+        <v>3000000</v>
+      </c>
+      <c r="C7" s="5" t="n">
+        <v>99999999</v>
+      </c>
+      <c r="D7" s="13" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="E7" s="5" t="n">
+        <v>923000</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A1:E1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>